<commit_message>
fix: close batch1 mapping audit gaps
</commit_message>
<xml_diff>
--- a/fixtures/mapping/fixture_mapping.xlsx
+++ b/fixtures/mapping/fixture_mapping.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">实体映射!$A$1:$D$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">属性映射!$A$1:$G$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">属性映射!$A$1:$G$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="true">关系映射!$A$1:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="true">本体参考!$A$1:$F$1</definedName>
   </definedNames>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="138">
   <si>
     <t>sourceId</t>
   </si>
@@ -311,34 +311,34 @@
     <t>nodeTypeCode</t>
   </si>
   <si>
+    <t>segmentDistance</t>
+  </si>
+  <si>
+    <t>magneticCourse</t>
+  </si>
+  <si>
+    <t>reverseMagneticCourse</t>
+  </si>
+  <si>
+    <t>airspaceName</t>
+  </si>
+  <si>
+    <t>airspaceTypeCode</t>
+  </si>
+  <si>
+    <t>airspaceTypeName</t>
+  </si>
+  <si>
+    <t>airspaceLowerLimit</t>
+  </si>
+  <si>
+    <t>airspaceUpperLimit</t>
+  </si>
+  <si>
     <t>sequenceNumber</t>
   </si>
   <si>
     <t>integer</t>
-  </si>
-  <si>
-    <t>segmentDistance</t>
-  </si>
-  <si>
-    <t>magneticCourse</t>
-  </si>
-  <si>
-    <t>reverseMagneticCourse</t>
-  </si>
-  <si>
-    <t>airspaceName</t>
-  </si>
-  <si>
-    <t>airspaceTypeCode</t>
-  </si>
-  <si>
-    <t>airspaceTypeName</t>
-  </si>
-  <si>
-    <t>airspaceLowerLimit</t>
-  </si>
-  <si>
-    <t>airspaceUpperLimit</t>
   </si>
   <si>
     <t>isEndRaw</t>
@@ -730,7 +730,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="18.0" customWidth="true"/>
@@ -1742,16 +1742,16 @@
         <v>43</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="F44" t="s" s="0">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="G44" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45">
@@ -1765,10 +1765,10 @@
         <v>43</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E45" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F45" t="s" s="0">
         <v>70</v>
@@ -1782,16 +1782,16 @@
         <v>20</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="F46" t="s" s="0">
         <v>70</v>
@@ -1811,10 +1811,10 @@
         <v>46</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F47" t="s" s="0">
         <v>70</v>
@@ -1834,10 +1834,10 @@
         <v>46</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F48" t="s" s="0">
         <v>70</v>
@@ -1851,22 +1851,22 @@
         <v>20</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F49" t="s" s="0">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="G49" t="s" s="0">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50">
@@ -1880,16 +1880,16 @@
         <v>49</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="F50" t="s" s="0">
         <v>63</v>
       </c>
       <c r="G50" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51">
@@ -1903,10 +1903,10 @@
         <v>49</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F51" t="s" s="0">
         <v>63</v>
@@ -1926,10 +1926,10 @@
         <v>49</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F52" t="s" s="0">
         <v>63</v>
@@ -1949,10 +1949,10 @@
         <v>49</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F53" t="s" s="0">
         <v>63</v>
@@ -1972,10 +1972,10 @@
         <v>49</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F54" t="s" s="0">
         <v>63</v>
@@ -1989,22 +1989,22 @@
         <v>20</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="C55" t="s" s="0">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="D55" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="E55" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="F55" t="s" s="0">
         <v>105</v>
       </c>
-      <c r="E55" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="F55" t="s" s="0">
-        <v>63</v>
-      </c>
       <c r="G55" t="s" s="0">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56">
@@ -2018,16 +2018,16 @@
         <v>55</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="F56" t="s" s="0">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="G56" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="57">
@@ -2041,10 +2041,10 @@
         <v>55</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F57" t="s" s="0">
         <v>70</v>
@@ -2064,13 +2064,13 @@
         <v>55</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>71</v>
+        <v>106</v>
       </c>
       <c r="F58" t="s" s="0">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="G58" t="s" s="0">
         <v>66</v>
@@ -2081,22 +2081,22 @@
         <v>20</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C59" t="s" s="0">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>106</v>
+        <v>59</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>106</v>
+        <v>59</v>
       </c>
       <c r="F59" t="s" s="0">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="G59" t="s" s="0">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="60">
@@ -2110,16 +2110,16 @@
         <v>58</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>59</v>
+        <v>108</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>59</v>
+        <v>108</v>
       </c>
       <c r="F60" t="s" s="0">
         <v>63</v>
       </c>
       <c r="G60" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="61">
@@ -2133,10 +2133,10 @@
         <v>58</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="F61" t="s" s="0">
         <v>63</v>
@@ -2156,10 +2156,10 @@
         <v>58</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="E62" t="s" s="0">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="F62" t="s" s="0">
         <v>63</v>
@@ -2179,10 +2179,10 @@
         <v>58</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E63" t="s" s="0">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F63" t="s" s="0">
         <v>63</v>
@@ -2196,22 +2196,22 @@
         <v>20</v>
       </c>
       <c r="B64" t="s" s="0">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C64" t="s" s="0">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D64" t="s" s="0">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="E64" t="s" s="0">
-        <v>112</v>
+        <v>62</v>
       </c>
       <c r="F64" t="s" s="0">
         <v>63</v>
       </c>
       <c r="G64" t="s" s="0">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65">
@@ -2225,16 +2225,16 @@
         <v>61</v>
       </c>
       <c r="D65" t="s" s="0">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E65" t="s" s="0">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F65" t="s" s="0">
         <v>63</v>
       </c>
       <c r="G65" t="s" s="0">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="66">
@@ -2248,10 +2248,10 @@
         <v>61</v>
       </c>
       <c r="D66" t="s" s="0">
-        <v>67</v>
+        <v>111</v>
       </c>
       <c r="E66" t="s" s="0">
-        <v>67</v>
+        <v>113</v>
       </c>
       <c r="F66" t="s" s="0">
         <v>63</v>
@@ -2271,10 +2271,10 @@
         <v>61</v>
       </c>
       <c r="D67" t="s" s="0">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E67" t="s" s="0">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F67" t="s" s="0">
         <v>63</v>
@@ -2283,31 +2283,8 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="B68" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="C68" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="D68" t="s" s="0">
-        <v>109</v>
-      </c>
-      <c r="E68" t="s" s="0">
-        <v>114</v>
-      </c>
-      <c r="F68" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="G68" t="s" s="0">
-        <v>66</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G68"/>
+  <autoFilter ref="A1:G67"/>
   <dataValidations count="2">
     <dataValidation type="list" sqref="F2:F1048576" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="无效值" error="请从下拉列表中选择允许的值">
       <formula1>"trim,upper,lower,integer,long,decimal,boolean"</formula1>

</xml_diff>